<commit_message>
Add initial Excel file for financial request testing
</commit_message>
<xml_diff>
--- a/bahan_keuangan/permohonan dana IPTI.xlsx
+++ b/bahan_keuangan/permohonan dana IPTI.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1601F0-C9EF-EF48-9202-BDCFEA87EC07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E17EA042-5736-1048-A0C5-D1AF7E0F670B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Permohonan Dana" sheetId="37" r:id="rId1"/>
@@ -53,7 +53,7 @@
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -62,12 +62,21 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-IKU LLDikti dan PT</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>IKU LLDikti dan PT</t>
         </r>
       </text>
     </comment>
@@ -1183,19 +1192,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="8"/>
       <name val="Times New Roman"/>
@@ -1275,6 +1271,19 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -2017,7 +2026,7 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="36" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="312">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2557,14 +2566,14 @@
     <xf numFmtId="166" fontId="24" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="38" fillId="5" borderId="47" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="47" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="38" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="36" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="38" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="36" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2615,19 +2624,19 @@
     <xf numFmtId="170" fontId="24" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="40" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="38" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="40" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="38" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="41" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="39" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2637,19 +2646,19 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="45" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="43" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="5" borderId="52" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2670,7 +2679,7 @@
     <xf numFmtId="170" fontId="24" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2698,16 +2707,58 @@
     <xf numFmtId="170" fontId="24" fillId="5" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="5" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="5" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2756,48 +2807,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2824,6 +2833,18 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2836,59 +2857,47 @@
     <xf numFmtId="0" fontId="18" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="22" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3216,18 +3225,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23" x14ac:dyDescent="0.2">
-      <c r="A1" s="274" t="s">
+      <c r="A1" s="254" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="275"/>
-      <c r="C1" s="275"/>
-      <c r="D1" s="275"/>
-      <c r="E1" s="275"/>
-      <c r="F1" s="275"/>
-      <c r="G1" s="275"/>
-      <c r="H1" s="275"/>
-      <c r="I1" s="275"/>
-      <c r="J1" s="276"/>
+      <c r="B1" s="255"/>
+      <c r="C1" s="255"/>
+      <c r="D1" s="255"/>
+      <c r="E1" s="255"/>
+      <c r="F1" s="255"/>
+      <c r="G1" s="255"/>
+      <c r="H1" s="255"/>
+      <c r="I1" s="255"/>
+      <c r="J1" s="256"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="155"/>
@@ -3241,15 +3250,15 @@
       <c r="J3" s="156"/>
     </row>
     <row r="4" spans="1:10" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="277"/>
-      <c r="B4" s="278"/>
-      <c r="C4" s="278"/>
-      <c r="D4" s="278"/>
-      <c r="E4" s="278"/>
-      <c r="F4" s="278"/>
-      <c r="G4" s="278"/>
-      <c r="H4" s="278"/>
-      <c r="I4" s="278"/>
+      <c r="A4" s="258"/>
+      <c r="B4" s="249"/>
+      <c r="C4" s="249"/>
+      <c r="D4" s="249"/>
+      <c r="E4" s="249"/>
+      <c r="F4" s="249"/>
+      <c r="G4" s="249"/>
+      <c r="H4" s="249"/>
+      <c r="I4" s="249"/>
       <c r="J4" s="156"/>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3262,14 +3271,14 @@
       <c r="C5" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="267" t="s">
+      <c r="D5" s="257" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="267"/>
-      <c r="F5" s="267"/>
-      <c r="G5" s="267"/>
-      <c r="H5" s="267"/>
-      <c r="I5" s="267"/>
+      <c r="E5" s="257"/>
+      <c r="F5" s="257"/>
+      <c r="G5" s="257"/>
+      <c r="H5" s="257"/>
+      <c r="I5" s="257"/>
       <c r="J5" s="156"/>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3282,14 +3291,14 @@
       <c r="C6" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="267" t="s">
+      <c r="D6" s="257" t="s">
         <v>224</v>
       </c>
-      <c r="E6" s="267"/>
-      <c r="F6" s="267"/>
-      <c r="G6" s="267"/>
-      <c r="H6" s="267"/>
-      <c r="I6" s="267"/>
+      <c r="E6" s="257"/>
+      <c r="F6" s="257"/>
+      <c r="G6" s="257"/>
+      <c r="H6" s="257"/>
+      <c r="I6" s="257"/>
       <c r="J6" s="156"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3302,25 +3311,25 @@
       <c r="C7" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="271" t="s">
+      <c r="D7" s="259" t="s">
         <v>225</v>
       </c>
-      <c r="E7" s="271"/>
-      <c r="F7" s="271"/>
-      <c r="G7" s="271"/>
-      <c r="H7" s="271"/>
-      <c r="I7" s="271"/>
+      <c r="E7" s="259"/>
+      <c r="F7" s="259"/>
+      <c r="G7" s="259"/>
+      <c r="H7" s="259"/>
+      <c r="I7" s="259"/>
       <c r="J7" s="156"/>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="157"/>
       <c r="B8" s="58"/>
-      <c r="D8" s="271"/>
-      <c r="E8" s="271"/>
-      <c r="F8" s="271"/>
-      <c r="G8" s="271"/>
-      <c r="H8" s="271"/>
-      <c r="I8" s="271"/>
+      <c r="D8" s="259"/>
+      <c r="E8" s="259"/>
+      <c r="F8" s="259"/>
+      <c r="G8" s="259"/>
+      <c r="H8" s="259"/>
+      <c r="I8" s="259"/>
       <c r="J8" s="156"/>
     </row>
     <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3333,14 +3342,14 @@
       <c r="C9" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="267" t="s">
+      <c r="D9" s="257" t="s">
         <v>226</v>
       </c>
-      <c r="E9" s="267"/>
-      <c r="F9" s="267"/>
-      <c r="G9" s="267"/>
-      <c r="H9" s="267"/>
-      <c r="I9" s="267"/>
+      <c r="E9" s="257"/>
+      <c r="F9" s="257"/>
+      <c r="G9" s="257"/>
+      <c r="H9" s="257"/>
+      <c r="I9" s="257"/>
       <c r="J9" s="156"/>
     </row>
     <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3353,14 +3362,14 @@
       <c r="C10" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="271" t="s">
+      <c r="D10" s="259" t="s">
         <v>227</v>
       </c>
-      <c r="E10" s="271"/>
-      <c r="F10" s="271"/>
-      <c r="G10" s="271"/>
-      <c r="H10" s="271"/>
-      <c r="I10" s="271"/>
+      <c r="E10" s="259"/>
+      <c r="F10" s="259"/>
+      <c r="G10" s="259"/>
+      <c r="H10" s="259"/>
+      <c r="I10" s="259"/>
       <c r="J10" s="156"/>
     </row>
     <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3373,14 +3382,14 @@
       <c r="C11" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="267" t="s">
+      <c r="D11" s="257" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="267"/>
-      <c r="F11" s="267"/>
-      <c r="G11" s="267"/>
-      <c r="H11" s="267"/>
-      <c r="I11" s="267"/>
+      <c r="E11" s="257"/>
+      <c r="F11" s="257"/>
+      <c r="G11" s="257"/>
+      <c r="H11" s="257"/>
+      <c r="I11" s="257"/>
       <c r="J11" s="159"/>
     </row>
     <row r="12" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3393,14 +3402,14 @@
       <c r="C12" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="272" t="s">
+      <c r="D12" s="260" t="s">
         <v>271</v>
       </c>
-      <c r="E12" s="271"/>
-      <c r="F12" s="271"/>
-      <c r="G12" s="271"/>
-      <c r="H12" s="271"/>
-      <c r="I12" s="271"/>
+      <c r="E12" s="259"/>
+      <c r="F12" s="259"/>
+      <c r="G12" s="259"/>
+      <c r="H12" s="259"/>
+      <c r="I12" s="259"/>
       <c r="J12" s="160"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3413,14 +3422,14 @@
       <c r="C13" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="267" t="s">
+      <c r="D13" s="257" t="s">
         <v>246</v>
       </c>
-      <c r="E13" s="267"/>
-      <c r="F13" s="267"/>
-      <c r="G13" s="267"/>
-      <c r="H13" s="267"/>
-      <c r="I13" s="267"/>
+      <c r="E13" s="257"/>
+      <c r="F13" s="257"/>
+      <c r="G13" s="257"/>
+      <c r="H13" s="257"/>
+      <c r="I13" s="257"/>
       <c r="J13" s="159"/>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3433,14 +3442,14 @@
       <c r="C14" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="273">
+      <c r="D14" s="261">
         <v>46182</v>
       </c>
-      <c r="E14" s="267"/>
-      <c r="F14" s="267"/>
-      <c r="G14" s="267"/>
-      <c r="H14" s="267"/>
-      <c r="I14" s="267"/>
+      <c r="E14" s="257"/>
+      <c r="F14" s="257"/>
+      <c r="G14" s="257"/>
+      <c r="H14" s="257"/>
+      <c r="I14" s="257"/>
       <c r="J14" s="161"/>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3453,14 +3462,14 @@
       <c r="C15" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="267" t="s">
+      <c r="D15" s="257" t="s">
         <v>272</v>
       </c>
-      <c r="E15" s="267"/>
-      <c r="F15" s="267"/>
-      <c r="G15" s="267"/>
-      <c r="H15" s="267"/>
-      <c r="I15" s="267"/>
+      <c r="E15" s="257"/>
+      <c r="F15" s="257"/>
+      <c r="G15" s="257"/>
+      <c r="H15" s="257"/>
+      <c r="I15" s="257"/>
       <c r="J15" s="161"/>
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3469,17 +3478,17 @@
       <c r="D16" s="58" t="s">
         <v>217</v>
       </c>
-      <c r="E16" s="270" t="str">
+      <c r="E16" s="262" t="str">
         <f>'Rincian Biaya'!B5</f>
         <v>Honorarium Narasumber/Pembahas</v>
       </c>
-      <c r="F16" s="270"/>
-      <c r="G16" s="270"/>
-      <c r="H16" s="268">
+      <c r="F16" s="262"/>
+      <c r="G16" s="262"/>
+      <c r="H16" s="252">
         <f>'Rincian Biaya'!M8</f>
         <v>2000000</v>
       </c>
-      <c r="I16" s="268"/>
+      <c r="I16" s="252"/>
       <c r="J16" s="161"/>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3488,17 +3497,17 @@
       <c r="D17" s="58" t="s">
         <v>218</v>
       </c>
-      <c r="E17" s="270" t="str">
+      <c r="E17" s="262" t="str">
         <f>'Rincian Biaya'!B10</f>
         <v>Honorarium Moderator</v>
       </c>
-      <c r="F17" s="270"/>
-      <c r="G17" s="270"/>
-      <c r="H17" s="268">
+      <c r="F17" s="262"/>
+      <c r="G17" s="262"/>
+      <c r="H17" s="252">
         <f>'Rincian Biaya'!M13</f>
         <v>700000</v>
       </c>
-      <c r="I17" s="268"/>
+      <c r="I17" s="252"/>
       <c r="J17" s="161"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -3507,17 +3516,17 @@
       <c r="D18" s="58" t="s">
         <v>219</v>
       </c>
-      <c r="E18" s="269" t="str">
+      <c r="E18" s="251" t="str">
         <f>'Rincian Biaya'!B15</f>
         <v xml:space="preserve"> Honorarium Panitia</v>
       </c>
-      <c r="F18" s="269"/>
-      <c r="G18" s="269"/>
-      <c r="H18" s="268">
+      <c r="F18" s="251"/>
+      <c r="G18" s="251"/>
+      <c r="H18" s="252">
         <f>'Rincian Biaya'!M24</f>
         <v>1175000</v>
       </c>
-      <c r="I18" s="268"/>
+      <c r="I18" s="252"/>
       <c r="J18" s="161"/>
     </row>
     <row r="19" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3530,17 +3539,17 @@
       <c r="D19" s="58" t="s">
         <v>220</v>
       </c>
-      <c r="E19" s="269" t="str">
+      <c r="E19" s="251" t="str">
         <f>'Rincian Biaya'!B26</f>
         <v>Transport Kegiatan Dalam Kota</v>
       </c>
-      <c r="F19" s="269"/>
-      <c r="G19" s="269"/>
-      <c r="H19" s="280">
+      <c r="F19" s="251"/>
+      <c r="G19" s="251"/>
+      <c r="H19" s="253">
         <f>'Rincian Biaya'!M34</f>
         <v>1020000</v>
       </c>
-      <c r="I19" s="280"/>
+      <c r="I19" s="253"/>
       <c r="J19" s="162"/>
     </row>
     <row r="20" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -3553,11 +3562,11 @@
         <f>'Rincian Biaya'!B36</f>
         <v>Uang Saku/ Uang Harian Kegiatan Dalam Kota</v>
       </c>
-      <c r="H20" s="268">
+      <c r="H20" s="252">
         <f>'Rincian Biaya'!M45</f>
         <v>910000</v>
       </c>
-      <c r="I20" s="268"/>
+      <c r="I20" s="252"/>
       <c r="J20" s="162"/>
     </row>
     <row r="21" spans="1:10" ht="35.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3566,17 +3575,17 @@
       <c r="D21" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="E21" s="269" t="str">
+      <c r="E21" s="251" t="str">
         <f>'Rincian Biaya'!B48</f>
         <v>Transport Kegiatan Dalam Kota Survei Lokasi Acara Kegiatan</v>
       </c>
-      <c r="F21" s="269"/>
-      <c r="G21" s="269"/>
-      <c r="H21" s="268">
+      <c r="F21" s="251"/>
+      <c r="G21" s="251"/>
+      <c r="H21" s="252">
         <f>'Rincian Biaya'!M52</f>
         <v>340000</v>
       </c>
-      <c r="I21" s="268"/>
+      <c r="I21" s="252"/>
       <c r="J21" s="162"/>
     </row>
     <row r="22" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3585,17 +3594,17 @@
       <c r="D22" s="58" t="s">
         <v>223</v>
       </c>
-      <c r="E22" s="269" t="str">
+      <c r="E22" s="251" t="str">
         <f>'Rincian Biaya'!B54</f>
         <v>Transport Kegiatan Dalam Kota Persiapan Akhir</v>
       </c>
-      <c r="F22" s="269"/>
-      <c r="G22" s="269"/>
-      <c r="H22" s="268">
+      <c r="F22" s="251"/>
+      <c r="G22" s="251"/>
+      <c r="H22" s="252">
         <f>'Rincian Biaya'!M58</f>
         <v>340000</v>
       </c>
-      <c r="I22" s="268"/>
+      <c r="I22" s="252"/>
       <c r="J22" s="162"/>
     </row>
     <row r="23" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3604,33 +3613,33 @@
       <c r="D23" s="58" t="s">
         <v>269</v>
       </c>
-      <c r="E23" s="269" t="str">
+      <c r="E23" s="251" t="str">
         <f>'Rincian Biaya'!B62</f>
         <v>Belanja Pendukung Lainnya (Belanja Bahan)</v>
       </c>
-      <c r="F23" s="269"/>
-      <c r="G23" s="269"/>
-      <c r="H23" s="268">
+      <c r="F23" s="251"/>
+      <c r="G23" s="251"/>
+      <c r="H23" s="252">
         <f>'Rincian Biaya'!F66</f>
         <v>24300000</v>
       </c>
-      <c r="I23" s="268"/>
+      <c r="I23" s="252"/>
       <c r="J23" s="162"/>
     </row>
     <row r="24" spans="1:10" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="157"/>
       <c r="B24" s="58"/>
       <c r="D24" s="58"/>
-      <c r="E24" s="278" t="s">
+      <c r="E24" s="249" t="s">
         <v>40</v>
       </c>
-      <c r="F24" s="278"/>
-      <c r="G24" s="278"/>
-      <c r="H24" s="279">
+      <c r="F24" s="249"/>
+      <c r="G24" s="249"/>
+      <c r="H24" s="250">
         <f>SUM(H16:I23)</f>
         <v>30785000</v>
       </c>
-      <c r="I24" s="279"/>
+      <c r="I24" s="250"/>
       <c r="J24" s="156"/>
     </row>
     <row r="25" spans="1:10" ht="30.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
@@ -3946,6 +3955,24 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="D15:I15"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="D14:I14"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="D7:I8"/>
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="E23:G23"/>
@@ -3957,71 +3984,16 @@
     <mergeCell ref="H19:I19"/>
     <mergeCell ref="E21:G21"/>
     <mergeCell ref="H21:I21"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="D6:I6"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="D9:I9"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="D7:I8"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="D13:I13"/>
-    <mergeCell ref="D14:I14"/>
-    <mergeCell ref="D15:I15"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E16:G16"/>
   </mergeCells>
-  <phoneticPr fontId="35" type="noConversion"/>
+  <phoneticPr fontId="33" type="noConversion"/>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:I6 D13:I13 H45 D9:I10 D7" xr:uid="{F2E9E5BB-EA0C-4733-B834-F4F8806AE5AE}">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="65" fitToHeight="0" orientation="portrait" useFirstPageNumber="1" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F2E9E5BB-EA0C-4733-B834-F4F8806AE5AE}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>D6:I6</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6FC5AC9C-370C-4ADC-834F-82D18CB530B9}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>D7</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FB3C639F-D8D3-4B31-85F7-D35A7A1871AC}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>D9:I9</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{43F96322-C905-4F01-B8AC-D9131C0C6A32}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>D10:I10</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5BE38D73-A111-475E-8644-C4F4AF882AFE}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>H45</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F819706B-61A9-492A-A5E3-8AFE66ED6667}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>D13:I13</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -4113,38 +4085,38 @@
       <c r="F8" s="281"/>
     </row>
     <row r="9" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="299"/>
-      <c r="B9" s="299"/>
-      <c r="C9" s="299"/>
-      <c r="D9" s="299"/>
-      <c r="E9" s="299"/>
-      <c r="F9" s="299"/>
+      <c r="A9" s="307"/>
+      <c r="B9" s="307"/>
+      <c r="C9" s="307"/>
+      <c r="D9" s="307"/>
+      <c r="E9" s="307"/>
+      <c r="F9" s="307"/>
     </row>
     <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="303" t="s">
+      <c r="A10" s="305" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="303" t="s">
+      <c r="B10" s="305" t="s">
         <v>76</v>
       </c>
       <c r="C10" s="308"/>
-      <c r="D10" s="305" t="s">
+      <c r="D10" s="300" t="s">
         <v>184</v>
       </c>
       <c r="E10" s="309" t="s">
         <v>185</v>
       </c>
-      <c r="F10" s="305" t="s">
+      <c r="F10" s="300" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="303"/>
-      <c r="B11" s="303"/>
+      <c r="A11" s="305"/>
+      <c r="B11" s="305"/>
       <c r="C11" s="308"/>
-      <c r="D11" s="305"/>
+      <c r="D11" s="300"/>
       <c r="E11" s="309"/>
-      <c r="F11" s="305"/>
+      <c r="F11" s="300"/>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="95" t="s">
@@ -4587,10 +4559,10 @@
       </c>
     </row>
     <row r="34" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="300" t="s">
+      <c r="A34" s="302" t="s">
         <v>175</v>
       </c>
-      <c r="B34" s="300"/>
+      <c r="B34" s="302"/>
       <c r="C34" s="103">
         <v>0</v>
       </c>
@@ -4605,26 +4577,26 @@
       <c r="M34" s="107"/>
     </row>
     <row r="35" spans="1:13" s="81" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="301" t="s">
+      <c r="A35" s="303" t="s">
         <v>103</v>
       </c>
-      <c r="B35" s="301"/>
-      <c r="C35" s="302" t="e">
+      <c r="B35" s="303"/>
+      <c r="C35" s="304" t="e">
         <v>#NAME?</v>
       </c>
-      <c r="D35" s="302"/>
-      <c r="E35" s="302"/>
-      <c r="F35" s="302"/>
+      <c r="D35" s="304"/>
+      <c r="E35" s="304"/>
+      <c r="F35" s="304"/>
       <c r="K35" s="108"/>
     </row>
     <row r="36" spans="1:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F36" s="109"/>
     </row>
     <row r="37" spans="1:13" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E37" s="270" t="s">
+      <c r="E37" s="262" t="s">
         <v>52</v>
       </c>
-      <c r="F37" s="270"/>
+      <c r="F37" s="262"/>
     </row>
     <row r="38" spans="1:13" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="85" t="s">
@@ -4645,10 +4617,10 @@
         <v>108</v>
       </c>
       <c r="D39" s="111"/>
-      <c r="E39" s="306" t="s">
+      <c r="E39" s="299" t="s">
         <v>109</v>
       </c>
-      <c r="F39" s="306"/>
+      <c r="F39" s="299"/>
     </row>
     <row r="40" spans="1:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="85" t="s">
@@ -4710,6 +4682,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A9:F9"/>
     <mergeCell ref="E39:F39"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="A34:B34"/>
@@ -4721,11 +4698,6 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="E10:E11"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A9:F9"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.49" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="85" orientation="portrait" useFirstPageNumber="1" horizontalDpi="120" verticalDpi="72"/>
@@ -4836,50 +4808,50 @@
       <c r="H9" s="281"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="299"/>
-      <c r="B10" s="299"/>
-      <c r="C10" s="299"/>
-      <c r="D10" s="299"/>
-      <c r="E10" s="299"/>
-      <c r="F10" s="299"/>
-      <c r="G10" s="299"/>
-      <c r="H10" s="299"/>
+      <c r="A10" s="307"/>
+      <c r="B10" s="307"/>
+      <c r="C10" s="307"/>
+      <c r="D10" s="307"/>
+      <c r="E10" s="307"/>
+      <c r="F10" s="307"/>
+      <c r="G10" s="307"/>
+      <c r="H10" s="307"/>
     </row>
     <row r="11" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="303" t="s">
+      <c r="A11" s="305" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="303" t="s">
+      <c r="B11" s="305" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="304" t="s">
+      <c r="C11" s="306" t="s">
         <v>192</v>
       </c>
-      <c r="D11" s="310" t="s">
+      <c r="D11" s="311" t="s">
         <v>193</v>
       </c>
-      <c r="E11" s="305" t="s">
+      <c r="E11" s="300" t="s">
         <v>194</v>
       </c>
-      <c r="F11" s="303" t="s">
+      <c r="F11" s="305" t="s">
         <v>195</v>
       </c>
-      <c r="G11" s="307" t="s">
+      <c r="G11" s="301" t="s">
         <v>196</v>
       </c>
-      <c r="H11" s="305" t="s">
+      <c r="H11" s="300" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="303"/>
-      <c r="B12" s="303"/>
-      <c r="C12" s="304"/>
-      <c r="D12" s="310"/>
-      <c r="E12" s="305"/>
-      <c r="F12" s="303"/>
-      <c r="G12" s="307"/>
-      <c r="H12" s="305"/>
+      <c r="A12" s="305"/>
+      <c r="B12" s="305"/>
+      <c r="C12" s="306"/>
+      <c r="D12" s="311"/>
+      <c r="E12" s="300"/>
+      <c r="F12" s="305"/>
+      <c r="G12" s="301"/>
+      <c r="H12" s="300"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="95" t="s">
@@ -5459,10 +5431,10 @@
       </c>
     </row>
     <row r="33" spans="1:15" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="300" t="s">
+      <c r="A33" s="302" t="s">
         <v>175</v>
       </c>
-      <c r="B33" s="300"/>
+      <c r="B33" s="302"/>
       <c r="C33" s="103">
         <f>SUM(C14:C32)</f>
         <v>19</v>
@@ -5488,28 +5460,28 @@
       <c r="O33" s="107"/>
     </row>
     <row r="34" spans="1:15" s="81" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="301" t="s">
+      <c r="A34" s="303" t="s">
         <v>103</v>
       </c>
-      <c r="B34" s="301"/>
-      <c r="C34" s="302" t="e">
+      <c r="B34" s="303"/>
+      <c r="C34" s="304" t="e">
         <v>#NAME?</v>
       </c>
-      <c r="D34" s="302"/>
-      <c r="E34" s="302"/>
-      <c r="F34" s="302"/>
-      <c r="G34" s="302"/>
-      <c r="H34" s="302"/>
+      <c r="D34" s="304"/>
+      <c r="E34" s="304"/>
+      <c r="F34" s="304"/>
+      <c r="G34" s="304"/>
+      <c r="H34" s="304"/>
       <c r="M34" s="108"/>
     </row>
     <row r="35" spans="1:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H35" s="109"/>
     </row>
     <row r="36" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G36" s="270" t="s">
+      <c r="G36" s="262" t="s">
         <v>207</v>
       </c>
-      <c r="H36" s="270"/>
+      <c r="H36" s="262"/>
     </row>
     <row r="37" spans="1:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="85" t="s">
@@ -5528,10 +5500,10 @@
         <v>108</v>
       </c>
       <c r="D38" s="115"/>
-      <c r="G38" s="296" t="s">
+      <c r="G38" s="292" t="s">
         <v>109</v>
       </c>
-      <c r="H38" s="296"/>
+      <c r="H38" s="292"/>
     </row>
     <row r="39" spans="1:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="85" t="s">
@@ -5565,14 +5537,14 @@
         <v>208</v>
       </c>
       <c r="B43" s="113"/>
-      <c r="C43" s="311" t="s">
+      <c r="C43" s="310" t="s">
         <v>147</v>
       </c>
-      <c r="D43" s="311"/>
-      <c r="G43" s="267" t="s">
+      <c r="D43" s="310"/>
+      <c r="G43" s="257" t="s">
         <v>5</v>
       </c>
-      <c r="H43" s="267"/>
+      <c r="H43" s="257"/>
     </row>
     <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="113" t="s">
@@ -5605,13 +5577,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A9:H9"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B11:B12"/>
@@ -5621,11 +5591,13 @@
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="G11:G12"/>
     <mergeCell ref="H11:H12"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G38:H38"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.49" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="85" orientation="portrait" useFirstPageNumber="1" horizontalDpi="120" verticalDpi="72"/>
@@ -5660,55 +5632,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="121" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="257" t="s">
+      <c r="A1" s="271" t="s">
         <v>228</v>
       </c>
-      <c r="B1" s="258"/>
-      <c r="C1" s="258"/>
-      <c r="D1" s="258"/>
-      <c r="E1" s="258"/>
-      <c r="F1" s="258"/>
-      <c r="G1" s="258"/>
-      <c r="H1" s="258"/>
-      <c r="I1" s="258"/>
-      <c r="J1" s="258"/>
-      <c r="K1" s="258"/>
-      <c r="L1" s="258"/>
-      <c r="M1" s="258"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="272"/>
+      <c r="G1" s="272"/>
+      <c r="H1" s="272"/>
+      <c r="I1" s="272"/>
+      <c r="J1" s="272"/>
+      <c r="K1" s="272"/>
+      <c r="L1" s="272"/>
+      <c r="M1" s="272"/>
     </row>
     <row r="2" spans="1:16" s="121" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="119"/>
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="273" t="s">
         <v>274</v>
       </c>
-      <c r="C2" s="259"/>
-      <c r="D2" s="259"/>
-      <c r="E2" s="259"/>
-      <c r="F2" s="259"/>
-      <c r="G2" s="259"/>
-      <c r="H2" s="259"/>
-      <c r="I2" s="259"/>
-      <c r="J2" s="259"/>
-      <c r="K2" s="259"/>
-      <c r="L2" s="259"/>
-      <c r="M2" s="259"/>
+      <c r="C2" s="273"/>
+      <c r="D2" s="273"/>
+      <c r="E2" s="273"/>
+      <c r="F2" s="273"/>
+      <c r="G2" s="273"/>
+      <c r="H2" s="273"/>
+      <c r="I2" s="273"/>
+      <c r="J2" s="273"/>
+      <c r="K2" s="273"/>
+      <c r="L2" s="273"/>
+      <c r="M2" s="273"/>
     </row>
     <row r="3" spans="1:16" s="121" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="119"/>
-      <c r="B3" s="266" t="s">
+      <c r="B3" s="280" t="s">
         <v>273</v>
       </c>
-      <c r="C3" s="266"/>
-      <c r="D3" s="266"/>
-      <c r="E3" s="266"/>
-      <c r="F3" s="266"/>
-      <c r="G3" s="266"/>
-      <c r="H3" s="266"/>
-      <c r="I3" s="266"/>
-      <c r="J3" s="266"/>
-      <c r="K3" s="266"/>
-      <c r="L3" s="266"/>
-      <c r="M3" s="266"/>
+      <c r="C3" s="280"/>
+      <c r="D3" s="280"/>
+      <c r="E3" s="280"/>
+      <c r="F3" s="280"/>
+      <c r="G3" s="280"/>
+      <c r="H3" s="280"/>
+      <c r="I3" s="280"/>
+      <c r="J3" s="280"/>
+      <c r="K3" s="280"/>
+      <c r="L3" s="280"/>
+      <c r="M3" s="280"/>
     </row>
     <row r="4" spans="1:16" s="121" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="119"/>
@@ -5831,17 +5803,17 @@
       </c>
     </row>
     <row r="8" spans="1:16" s="122" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="254" t="s">
+      <c r="A8" s="268" t="s">
         <v>175</v>
       </c>
-      <c r="B8" s="255"/>
-      <c r="C8" s="255"/>
-      <c r="D8" s="255"/>
-      <c r="E8" s="255"/>
-      <c r="F8" s="255"/>
-      <c r="G8" s="255"/>
-      <c r="H8" s="255"/>
-      <c r="I8" s="256"/>
+      <c r="B8" s="269"/>
+      <c r="C8" s="269"/>
+      <c r="D8" s="269"/>
+      <c r="E8" s="269"/>
+      <c r="F8" s="269"/>
+      <c r="G8" s="269"/>
+      <c r="H8" s="269"/>
+      <c r="I8" s="270"/>
       <c r="J8" s="175"/>
       <c r="K8" s="176"/>
       <c r="L8" s="177"/>
@@ -5977,17 +5949,17 @@
       <c r="P12" s="196"/>
     </row>
     <row r="13" spans="1:16" s="195" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="264" t="s">
+      <c r="A13" s="278" t="s">
         <v>175</v>
       </c>
-      <c r="B13" s="265"/>
-      <c r="C13" s="265"/>
-      <c r="D13" s="265"/>
-      <c r="E13" s="265"/>
-      <c r="F13" s="265"/>
-      <c r="G13" s="265"/>
-      <c r="H13" s="265"/>
-      <c r="I13" s="265"/>
+      <c r="B13" s="279"/>
+      <c r="C13" s="279"/>
+      <c r="D13" s="279"/>
+      <c r="E13" s="279"/>
+      <c r="F13" s="279"/>
+      <c r="G13" s="279"/>
+      <c r="H13" s="279"/>
+      <c r="I13" s="279"/>
       <c r="J13" s="200"/>
       <c r="K13" s="201"/>
       <c r="L13" s="202"/>
@@ -6389,17 +6361,17 @@
       </c>
     </row>
     <row r="24" spans="1:16" s="122" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="252" t="s">
+      <c r="A24" s="266" t="s">
         <v>175</v>
       </c>
-      <c r="B24" s="253"/>
-      <c r="C24" s="253"/>
-      <c r="D24" s="253"/>
-      <c r="E24" s="253"/>
-      <c r="F24" s="253"/>
-      <c r="G24" s="253"/>
-      <c r="H24" s="253"/>
-      <c r="I24" s="253"/>
+      <c r="B24" s="267"/>
+      <c r="C24" s="267"/>
+      <c r="D24" s="267"/>
+      <c r="E24" s="267"/>
+      <c r="F24" s="267"/>
+      <c r="G24" s="267"/>
+      <c r="H24" s="267"/>
+      <c r="I24" s="267"/>
       <c r="J24" s="232"/>
       <c r="K24" s="233"/>
       <c r="L24" s="234"/>
@@ -6759,17 +6731,17 @@
       <c r="P33" s="174"/>
     </row>
     <row r="34" spans="1:16" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="263" t="s">
+      <c r="A34" s="277" t="s">
         <v>175</v>
       </c>
-      <c r="B34" s="263"/>
-      <c r="C34" s="263"/>
-      <c r="D34" s="263"/>
-      <c r="E34" s="263"/>
-      <c r="F34" s="263"/>
-      <c r="G34" s="263"/>
-      <c r="H34" s="263"/>
-      <c r="I34" s="263"/>
+      <c r="B34" s="277"/>
+      <c r="C34" s="277"/>
+      <c r="D34" s="277"/>
+      <c r="E34" s="277"/>
+      <c r="F34" s="277"/>
+      <c r="G34" s="277"/>
+      <c r="H34" s="277"/>
+      <c r="I34" s="277"/>
       <c r="J34" s="175"/>
       <c r="K34" s="176"/>
       <c r="L34" s="177"/>
@@ -7169,17 +7141,17 @@
       </c>
     </row>
     <row r="45" spans="1:16" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="263" t="s">
+      <c r="A45" s="277" t="s">
         <v>175</v>
       </c>
-      <c r="B45" s="263"/>
-      <c r="C45" s="263"/>
-      <c r="D45" s="263"/>
-      <c r="E45" s="263"/>
-      <c r="F45" s="263"/>
-      <c r="G45" s="263"/>
-      <c r="H45" s="263"/>
-      <c r="I45" s="263"/>
+      <c r="B45" s="277"/>
+      <c r="C45" s="277"/>
+      <c r="D45" s="277"/>
+      <c r="E45" s="277"/>
+      <c r="F45" s="277"/>
+      <c r="G45" s="277"/>
+      <c r="H45" s="277"/>
+      <c r="I45" s="277"/>
       <c r="J45" s="175"/>
       <c r="K45" s="147"/>
       <c r="L45" s="148"/>
@@ -7355,17 +7327,17 @@
       </c>
     </row>
     <row r="52" spans="1:17" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="260" t="s">
+      <c r="A52" s="274" t="s">
         <v>175</v>
       </c>
-      <c r="B52" s="261"/>
-      <c r="C52" s="261"/>
-      <c r="D52" s="261"/>
-      <c r="E52" s="261"/>
-      <c r="F52" s="261"/>
-      <c r="G52" s="261"/>
-      <c r="H52" s="261"/>
-      <c r="I52" s="262"/>
+      <c r="B52" s="275"/>
+      <c r="C52" s="275"/>
+      <c r="D52" s="275"/>
+      <c r="E52" s="275"/>
+      <c r="F52" s="275"/>
+      <c r="G52" s="275"/>
+      <c r="H52" s="275"/>
+      <c r="I52" s="276"/>
       <c r="J52" s="175"/>
       <c r="K52" s="176"/>
       <c r="L52" s="177"/>
@@ -7540,17 +7512,17 @@
       </c>
     </row>
     <row r="58" spans="1:17" s="180" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="260" t="s">
+      <c r="A58" s="274" t="s">
         <v>175</v>
       </c>
-      <c r="B58" s="261"/>
-      <c r="C58" s="261"/>
-      <c r="D58" s="261"/>
-      <c r="E58" s="261"/>
-      <c r="F58" s="261"/>
-      <c r="G58" s="261"/>
-      <c r="H58" s="261"/>
-      <c r="I58" s="262"/>
+      <c r="B58" s="275"/>
+      <c r="C58" s="275"/>
+      <c r="D58" s="275"/>
+      <c r="E58" s="275"/>
+      <c r="F58" s="275"/>
+      <c r="G58" s="275"/>
+      <c r="H58" s="275"/>
+      <c r="I58" s="276"/>
       <c r="J58" s="175"/>
       <c r="K58" s="176"/>
       <c r="L58" s="177"/>
@@ -7664,13 +7636,13 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="249" t="s">
+      <c r="A66" s="263" t="s">
         <v>175</v>
       </c>
-      <c r="B66" s="250"/>
-      <c r="C66" s="250"/>
-      <c r="D66" s="250"/>
-      <c r="E66" s="251"/>
+      <c r="B66" s="264"/>
+      <c r="C66" s="264"/>
+      <c r="D66" s="264"/>
+      <c r="E66" s="265"/>
       <c r="F66" s="229">
         <f>SUM(F64:F65)</f>
         <v>24300000</v>
@@ -7697,26 +7669,13 @@
     <mergeCell ref="B3:M3"/>
     <mergeCell ref="A58:I58"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B60:C60 B7:C7 B17:C23 B50:C51 B56:C57 B12 B28:C33 B38:C44" xr:uid="{F7D5BBFD-630D-408A-BB88-16A273EE465C}">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.43307086614173229" right="0.35433070866141736" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="60" fitToHeight="0" orientation="landscape" useFirstPageNumber="1" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F7D5BBFD-630D-408A-BB88-16A273EE465C}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>C60 C7 C17:C23 C28:C33 C50:C51 C56:C57 C38:C44</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D56B2F79-BB30-4171-814D-7BF4ACA8AC23}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>B60 B7 B17:B23 B50:B51 B56:B57 B12 B28:B33 B38:B44</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -8846,39 +8805,39 @@
       <c r="H9" s="65"/>
     </row>
     <row r="10" spans="1:11" s="66" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="292" t="s">
+      <c r="A10" s="296" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="292" t="s">
+      <c r="B10" s="296" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="292" t="s">
+      <c r="C10" s="296" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="293" t="s">
+      <c r="D10" s="297" t="s">
         <v>77</v>
       </c>
-      <c r="E10" s="290" t="s">
+      <c r="E10" s="294" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="290"/>
-      <c r="G10" s="290"/>
-      <c r="H10" s="291" t="s">
+      <c r="F10" s="294"/>
+      <c r="G10" s="294"/>
+      <c r="H10" s="295" t="s">
         <v>79</v>
       </c>
-      <c r="I10" s="291"/>
-      <c r="J10" s="293" t="s">
+      <c r="I10" s="295"/>
+      <c r="J10" s="297" t="s">
         <v>80</v>
       </c>
-      <c r="K10" s="292" t="s">
+      <c r="K10" s="296" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="66" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="292"/>
-      <c r="B11" s="292"/>
-      <c r="C11" s="292"/>
-      <c r="D11" s="293"/>
+      <c r="A11" s="296"/>
+      <c r="B11" s="296"/>
+      <c r="C11" s="296"/>
+      <c r="D11" s="297"/>
       <c r="E11" s="67" t="s">
         <v>132</v>
       </c>
@@ -8894,8 +8853,8 @@
       <c r="I11" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="J11" s="293"/>
-      <c r="K11" s="292"/>
+      <c r="J11" s="297"/>
+      <c r="K11" s="296"/>
     </row>
     <row r="12" spans="1:11" s="66" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="68" t="s">
@@ -9118,10 +9077,10 @@
       <c r="K17" s="68"/>
     </row>
     <row r="18" spans="1:11" s="81" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="294" t="s">
+      <c r="A18" s="290" t="s">
         <v>103</v>
       </c>
-      <c r="B18" s="294"/>
+      <c r="B18" s="290"/>
       <c r="C18" s="82" t="e">
         <v>#NAME?</v>
       </c>
@@ -9142,10 +9101,10 @@
     </row>
     <row r="21" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="22" spans="1:11" ht="14" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="J22" s="295" t="s">
+      <c r="J22" s="291" t="s">
         <v>145</v>
       </c>
-      <c r="K22" s="295"/>
+      <c r="K22" s="291"/>
     </row>
     <row r="23" spans="1:11" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="85" t="s">
@@ -9164,10 +9123,10 @@
       <c r="E24" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="J24" s="296" t="s">
+      <c r="J24" s="292" t="s">
         <v>109</v>
       </c>
-      <c r="K24" s="296"/>
+      <c r="K24" s="292"/>
     </row>
     <row r="25" spans="1:11" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="85" t="s">
@@ -9197,14 +9156,14 @@
       <c r="A29" s="87" t="s">
         <v>146</v>
       </c>
-      <c r="E29" s="297" t="s">
+      <c r="E29" s="293" t="s">
         <v>147</v>
       </c>
-      <c r="F29" s="297"/>
-      <c r="J29" s="297" t="s">
+      <c r="F29" s="293"/>
+      <c r="J29" s="293" t="s">
         <v>148</v>
       </c>
-      <c r="K29" s="297"/>
+      <c r="K29" s="293"/>
     </row>
     <row r="30" spans="1:11" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="87" t="s">
@@ -9221,11 +9180,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="J29:K29"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A6:K6"/>
     <mergeCell ref="A7:K7"/>
@@ -9238,6 +9192,11 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="J10:J11"/>
     <mergeCell ref="K10:K11"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="J29:K29"/>
   </mergeCells>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.59055118110236227" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="95" orientation="landscape" useFirstPageNumber="1" horizontalDpi="120" verticalDpi="72"/>
@@ -10516,48 +10475,48 @@
       <c r="H8" s="281"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="299"/>
-      <c r="B9" s="299"/>
-      <c r="C9" s="299"/>
-      <c r="D9" s="299"/>
-      <c r="E9" s="299"/>
-      <c r="F9" s="299"/>
-      <c r="G9" s="299"/>
-      <c r="H9" s="299"/>
+      <c r="A9" s="307"/>
+      <c r="B9" s="307"/>
+      <c r="C9" s="307"/>
+      <c r="D9" s="307"/>
+      <c r="E9" s="307"/>
+      <c r="F9" s="307"/>
+      <c r="G9" s="307"/>
+      <c r="H9" s="307"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="303" t="s">
+      <c r="A10" s="305" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="303" t="s">
+      <c r="B10" s="305" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="304" t="s">
+      <c r="C10" s="306" t="s">
         <v>169</v>
       </c>
-      <c r="D10" s="305"/>
-      <c r="E10" s="305" t="s">
+      <c r="D10" s="300"/>
+      <c r="E10" s="300" t="s">
         <v>170</v>
       </c>
-      <c r="F10" s="305" t="s">
+      <c r="F10" s="300" t="s">
         <v>171</v>
       </c>
-      <c r="G10" s="307" t="s">
+      <c r="G10" s="301" t="s">
         <v>172</v>
       </c>
-      <c r="H10" s="305" t="s">
+      <c r="H10" s="300" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="303"/>
-      <c r="B11" s="303"/>
-      <c r="C11" s="304"/>
-      <c r="D11" s="305"/>
-      <c r="E11" s="305"/>
-      <c r="F11" s="305"/>
-      <c r="G11" s="307"/>
-      <c r="H11" s="305"/>
+      <c r="A11" s="305"/>
+      <c r="B11" s="305"/>
+      <c r="C11" s="306"/>
+      <c r="D11" s="300"/>
+      <c r="E11" s="300"/>
+      <c r="F11" s="300"/>
+      <c r="G11" s="301"/>
+      <c r="H11" s="300"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="95" t="s">
@@ -11153,10 +11112,10 @@
       </c>
     </row>
     <row r="34" spans="1:15" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="300" t="s">
+      <c r="A34" s="302" t="s">
         <v>175</v>
       </c>
-      <c r="B34" s="300"/>
+      <c r="B34" s="302"/>
       <c r="C34" s="103">
         <v>0</v>
       </c>
@@ -11177,28 +11136,28 @@
       <c r="O34" s="107"/>
     </row>
     <row r="35" spans="1:15" s="81" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="301" t="s">
+      <c r="A35" s="303" t="s">
         <v>103</v>
       </c>
-      <c r="B35" s="301"/>
-      <c r="C35" s="302" t="e">
+      <c r="B35" s="303"/>
+      <c r="C35" s="304" t="e">
         <v>#NAME?</v>
       </c>
-      <c r="D35" s="302"/>
-      <c r="E35" s="302"/>
-      <c r="F35" s="302"/>
-      <c r="G35" s="302"/>
-      <c r="H35" s="302"/>
+      <c r="D35" s="304"/>
+      <c r="E35" s="304"/>
+      <c r="F35" s="304"/>
+      <c r="G35" s="304"/>
+      <c r="H35" s="304"/>
       <c r="M35" s="108"/>
     </row>
     <row r="36" spans="1:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H36" s="109"/>
     </row>
     <row r="37" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G37" s="270" t="s">
+      <c r="G37" s="262" t="s">
         <v>52</v>
       </c>
-      <c r="H37" s="270"/>
+      <c r="H37" s="262"/>
     </row>
     <row r="38" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="85" t="s">
@@ -11223,10 +11182,10 @@
       </c>
       <c r="E39" s="112"/>
       <c r="F39" s="112"/>
-      <c r="G39" s="306" t="s">
+      <c r="G39" s="299" t="s">
         <v>109</v>
       </c>
-      <c r="H39" s="306"/>
+      <c r="H39" s="299"/>
     </row>
     <row r="40" spans="1:15" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="85" t="s">
@@ -11317,11 +11276,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A9:H9"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="C35:H35"/>
@@ -11330,11 +11289,11 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="E10:E11"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H10:H11"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.49" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="85" orientation="portrait" useFirstPageNumber="1" horizontalDpi="120" verticalDpi="72"/>
@@ -11423,40 +11382,40 @@
       <c r="F8" s="281"/>
     </row>
     <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="299"/>
-      <c r="B9" s="299"/>
-      <c r="C9" s="299"/>
-      <c r="D9" s="299"/>
-      <c r="E9" s="299"/>
-      <c r="F9" s="299"/>
+      <c r="A9" s="307"/>
+      <c r="B9" s="307"/>
+      <c r="C9" s="307"/>
+      <c r="D9" s="307"/>
+      <c r="E9" s="307"/>
+      <c r="F9" s="307"/>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="303" t="s">
+      <c r="A10" s="305" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="303" t="s">
+      <c r="B10" s="305" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="304" t="s">
+      <c r="C10" s="306" t="s">
         <v>169</v>
       </c>
-      <c r="D10" s="305" t="s">
+      <c r="D10" s="300" t="s">
         <v>171</v>
       </c>
-      <c r="E10" s="307" t="s">
+      <c r="E10" s="301" t="s">
         <v>172</v>
       </c>
-      <c r="F10" s="305" t="s">
+      <c r="F10" s="300" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="303"/>
-      <c r="B11" s="303"/>
-      <c r="C11" s="304"/>
-      <c r="D11" s="305"/>
-      <c r="E11" s="307"/>
-      <c r="F11" s="305"/>
+      <c r="A11" s="305"/>
+      <c r="B11" s="305"/>
+      <c r="C11" s="306"/>
+      <c r="D11" s="300"/>
+      <c r="E11" s="301"/>
+      <c r="F11" s="300"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="95" t="s">
@@ -11902,10 +11861,10 @@
       </c>
     </row>
     <row r="34" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="300" t="s">
+      <c r="A34" s="302" t="s">
         <v>175</v>
       </c>
-      <c r="B34" s="300"/>
+      <c r="B34" s="302"/>
       <c r="C34" s="103">
         <v>6</v>
       </c>
@@ -11920,26 +11879,26 @@
       <c r="M34" s="107"/>
     </row>
     <row r="35" spans="1:13" s="81" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="301" t="s">
+      <c r="A35" s="303" t="s">
         <v>103</v>
       </c>
-      <c r="B35" s="301"/>
-      <c r="C35" s="302" t="e">
+      <c r="B35" s="303"/>
+      <c r="C35" s="304" t="e">
         <v>#NAME?</v>
       </c>
-      <c r="D35" s="302"/>
-      <c r="E35" s="302"/>
-      <c r="F35" s="302"/>
+      <c r="D35" s="304"/>
+      <c r="E35" s="304"/>
+      <c r="F35" s="304"/>
       <c r="K35" s="108"/>
     </row>
     <row r="36" spans="1:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F36" s="109"/>
     </row>
     <row r="37" spans="1:13" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E37" s="270" t="s">
+      <c r="E37" s="262" t="s">
         <v>52</v>
       </c>
-      <c r="F37" s="270"/>
+      <c r="F37" s="262"/>
     </row>
     <row r="38" spans="1:13" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="85" t="s">
@@ -11960,10 +11919,10 @@
         <v>108</v>
       </c>
       <c r="D39" s="111"/>
-      <c r="E39" s="306" t="s">
+      <c r="E39" s="299" t="s">
         <v>109</v>
       </c>
-      <c r="F39" s="306"/>
+      <c r="F39" s="299"/>
     </row>
     <row r="40" spans="1:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="85" t="s">
@@ -12025,6 +11984,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A9:F9"/>
     <mergeCell ref="E39:F39"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="A34:B34"/>
@@ -12036,11 +12000,6 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="E10:E11"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A9:F9"/>
   </mergeCells>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.49" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="85" orientation="portrait" useFirstPageNumber="1" horizontalDpi="120" verticalDpi="72"/>

</xml_diff>